<commit_message>
Working on a new test for simple neighbors.
</commit_message>
<xml_diff>
--- a/SimulationEngine/SimulationEngine/NeighborTest.xlsx
+++ b/SimulationEngine/SimulationEngine/NeighborTest.xlsx
@@ -1,23 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\6-Courses\19-ModernC++Projects\SimulationEngine\SimulationEngine\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{09AD373A-6EC7-4C64-B4CE-C4EC3655B59A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C50483B5-E871-49E8-ACCC-82301BC759E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6780" yWindow="732" windowWidth="17280" windowHeight="8880" xr2:uid="{D5DDC3B4-E262-4B33-B762-D227AD5ACECE}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{D5DDC3B4-E262-4B33-B762-D227AD5ACECE}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="test1" sheetId="1" r:id="rId1"/>
+    <sheet name="test2" sheetId="3" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="DIST">_xlfn.LAMBDA(_xlpm.x,_xlpm.y,SQRT((INDEX(Sheet1!$B$2:$D$11,_xlpm.x,1)-INDEX(Sheet1!$B$2:$D$11,_xlpm.y,1))^2+(INDEX(Sheet1!$B$2:$D$11,_xlpm.x,2)-INDEX(Sheet1!$B$2:$D$11,_xlpm.y,2))^2 +(INDEX(Sheet1!$B$2:$D$11,_xlpm.x,3)-INDEX(Sheet1!$B$2:$D$11,_xlpm.y,3))^2) )</definedName>
-    <definedName name="DISTANCE" localSheetId="0">Sheet1!$E$15</definedName>
+    <definedName name="DIST" localSheetId="1">_xlfn.LAMBDA(_xlpm.x,_xlpm.y,SQRT((INDEX(test2!$B$2:$D$11,_xlpm.x,1)-INDEX(test2!$B$2:$D$11,_xlpm.y,1))^2+(INDEX(test2!$B$2:$D$11,_xlpm.x,2)-INDEX(test2!$B$2:$D$11,_xlpm.y,2))^2 +(INDEX(test2!$B$2:$D$11,_xlpm.x,3)-INDEX(test2!$B$2:$D$11,_xlpm.y,3))^2) )</definedName>
+    <definedName name="DIST">_xlfn.LAMBDA(_xlpm.x,_xlpm.y,SQRT((INDEX(test1!$B$2:$D$11,_xlpm.x,1)-INDEX(test1!$B$2:$D$11,_xlpm.y,1))^2+(INDEX(test1!$B$2:$D$11,_xlpm.x,2)-INDEX(test1!$B$2:$D$11,_xlpm.y,2))^2 +(INDEX(test1!$B$2:$D$11,_xlpm.x,3)-INDEX(test1!$B$2:$D$11,_xlpm.y,3))^2) )</definedName>
+    <definedName name="DISTANCE" localSheetId="0">test1!$E$15</definedName>
+    <definedName name="DISTANCE" localSheetId="1">test2!$E$15</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -77,7 +80,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="3">
   <si>
     <t>x</t>
   </si>
@@ -959,4 +962,451 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F835845-E7D8-43A5-A30F-70FD886764B4}">
+  <dimension ref="A1:P15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="G1">
+        <v>1</v>
+      </c>
+      <c r="H1">
+        <v>2</v>
+      </c>
+      <c r="I1">
+        <v>3</v>
+      </c>
+      <c r="J1">
+        <v>4</v>
+      </c>
+      <c r="K1">
+        <v>5</v>
+      </c>
+      <c r="L1">
+        <v>6</v>
+      </c>
+      <c r="M1">
+        <v>7</v>
+      </c>
+      <c r="N1">
+        <v>8</v>
+      </c>
+      <c r="O1">
+        <v>9</v>
+      </c>
+      <c r="P1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>-280</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2" cm="1">
+        <f t="array" ref="H2">IF(DIST(H$1,$F2)&lt;$H$13,1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="I2" cm="1">
+        <f t="array" ref="I2">IF(DIST(I$1,$F2)&lt;$H$13,1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="J2" cm="1">
+        <f t="array" ref="J2">IF(DIST(J$1,$F2)&lt;$H$13,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K2" cm="1">
+        <f t="array" ref="K2">IF(DIST(K$1,$F2)&lt;$H$13,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L2" cm="1">
+        <f t="array" ref="L2">IF(DIST(L$1,$F2)&lt;$H$13,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="M2" cm="1">
+        <f t="array" ref="M2">IF(DIST(M$1,$F2)&lt;$H$13,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="N2" cm="1">
+        <f t="array" ref="N2">IF(DIST(N$1,$F2)&lt;$H$13,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="O2" cm="1">
+        <f t="array" ref="O2">IF(DIST(O$1,$F2)&lt;$H$13,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="P2" cm="1">
+        <f t="array" ref="P2">IF(DIST(P$1,$F2)&lt;$H$13,1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>-260</v>
+      </c>
+      <c r="C3">
+        <v>5</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>2</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3" cm="1">
+        <f t="array" ref="I3">IF(DIST(I$1,$F3)&lt;$H$13,1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="J3" cm="1">
+        <f t="array" ref="J3">IF(DIST(J$1,$F3)&lt;$H$13,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K3" cm="1">
+        <f t="array" ref="K3">IF(DIST(K$1,$F3)&lt;$H$13,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L3" cm="1">
+        <f t="array" ref="L3">IF(DIST(L$1,$F3)&lt;$H$13,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="M3" cm="1">
+        <f t="array" ref="M3">IF(DIST(M$1,$F3)&lt;$H$13,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="N3" cm="1">
+        <f t="array" ref="N3">IF(DIST(N$1,$F3)&lt;$H$13,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="O3" cm="1">
+        <f t="array" ref="O3">IF(DIST(O$1,$F3)&lt;$H$13,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="P3" cm="1">
+        <f t="array" ref="P3">IF(DIST(P$1,$F3)&lt;$H$13,1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4">
+        <v>-240</v>
+      </c>
+      <c r="C4">
+        <v>-5</v>
+      </c>
+      <c r="D4">
+        <v>10</v>
+      </c>
+      <c r="F4">
+        <v>3</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4" cm="1">
+        <f t="array" ref="J4">IF(DIST(J$1,$F4)&lt;$H$13,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K4" cm="1">
+        <f t="array" ref="K4">IF(DIST(K$1,$F4)&lt;$H$13,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L4" cm="1">
+        <f t="array" ref="L4">IF(DIST(L$1,$F4)&lt;$H$13,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="M4" cm="1">
+        <f t="array" ref="M4">IF(DIST(M$1,$F4)&lt;$H$13,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="N4" cm="1">
+        <f t="array" ref="N4">IF(DIST(N$1,$F4)&lt;$H$13,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="O4" cm="1">
+        <f t="array" ref="O4">IF(DIST(O$1,$F4)&lt;$H$13,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="P4" cm="1">
+        <f t="array" ref="P4">IF(DIST(P$1,$F4)&lt;$H$13,1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5">
+        <v>-50</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>4</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5" cm="1">
+        <f t="array" ref="K5">IF(DIST(K$1,$F5)&lt;$H$13,1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="L5" cm="1">
+        <f t="array" ref="L5">IF(DIST(L$1,$F5)&lt;$H$13,1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="M5" cm="1">
+        <f t="array" ref="M5">IF(DIST(M$1,$F5)&lt;$H$13,1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="N5" cm="1">
+        <f t="array" ref="N5">IF(DIST(N$1,$F5)&lt;$H$13,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="O5" cm="1">
+        <f t="array" ref="O5">IF(DIST(O$1,$F5)&lt;$H$13,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="P5" cm="1">
+        <f t="array" ref="P5">IF(DIST(P$1,$F5)&lt;$H$13,1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>4</v>
+      </c>
+      <c r="B6">
+        <v>-30</v>
+      </c>
+      <c r="C6">
+        <v>10</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>5</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6" cm="1">
+        <f t="array" ref="L6">IF(DIST(L$1,$F6)&lt;$H$13,1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="M6" cm="1">
+        <f t="array" ref="M6">IF(DIST(M$1,$F6)&lt;$H$13,1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="N6" cm="1">
+        <f t="array" ref="N6">IF(DIST(N$1,$F6)&lt;$H$13,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="O6" cm="1">
+        <f t="array" ref="O6">IF(DIST(O$1,$F6)&lt;$H$13,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="P6" cm="1">
+        <f t="array" ref="P6">IF(DIST(P$1,$F6)&lt;$H$13,1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>5</v>
+      </c>
+      <c r="B7">
+        <v>-10</v>
+      </c>
+      <c r="C7">
+        <v>-5</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>6</v>
+      </c>
+      <c r="L7">
+        <v>0</v>
+      </c>
+      <c r="M7" cm="1">
+        <f t="array" ref="M7">IF(DIST(M$1,$F7)&lt;$H$13,1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="N7" cm="1">
+        <f t="array" ref="N7">IF(DIST(N$1,$F7)&lt;$H$13,1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="O7" cm="1">
+        <f t="array" ref="O7">IF(DIST(O$1,$F7)&lt;$H$13,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="P7" cm="1">
+        <f t="array" ref="P7">IF(DIST(P$1,$F7)&lt;$H$13,1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>6</v>
+      </c>
+      <c r="B8">
+        <v>15</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8">
+        <v>5</v>
+      </c>
+      <c r="F8">
+        <v>7</v>
+      </c>
+      <c r="M8">
+        <v>0</v>
+      </c>
+      <c r="N8" cm="1">
+        <f t="array" ref="N8">IF(DIST(N$1,$F8)&lt;$H$13,1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="O8" cm="1">
+        <f t="array" ref="O8">IF(DIST(O$1,$F8)&lt;$H$13,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="P8" cm="1">
+        <f t="array" ref="P8">IF(DIST(P$1,$F8)&lt;$H$13,1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>7</v>
+      </c>
+      <c r="B9">
+        <v>40</v>
+      </c>
+      <c r="C9">
+        <v>-5</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>8</v>
+      </c>
+      <c r="N9">
+        <v>0</v>
+      </c>
+      <c r="O9" cm="1">
+        <f t="array" ref="O9">IF(DIST(O$1,$F9)&lt;$H$13,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="P9" cm="1">
+        <f t="array" ref="P9">IF(DIST(P$1,$F9)&lt;$H$13,1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>8</v>
+      </c>
+      <c r="B10">
+        <v>200</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>9</v>
+      </c>
+      <c r="O10">
+        <v>0</v>
+      </c>
+      <c r="P10" cm="1">
+        <f t="array" ref="P10">IF(DIST(P$1,$F10)&lt;$H$13,1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>9</v>
+      </c>
+      <c r="B11">
+        <v>235</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="F11">
+        <v>10</v>
+      </c>
+      <c r="P11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="H13">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="E15" t="e" cm="1" vm="1">
+        <f t="array" ref="E15">_xlfn.LAMBDA(_xlpm.x,_xlpm.y,SQRT((INDEX($B$2:$D$11,_xlpm.x,1)-INDEX($B$2:$D$11,_xlpm.y,1))^2+(INDEX($B$2:$D$11,_xlpm.x,2)-INDEX($B$2:$D$11,_xlpm.y,2))^2 +(INDEX($B$2:$D$11,_xlpm.x,3)-INDEX($B$2:$D$11,_xlpm.y,3))^2)
+)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="H15" cm="1">
+        <f t="array" ref="H15">DIST(1,2)</f>
+        <v>20.615528128088304</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
passed the neighbor list test
</commit_message>
<xml_diff>
--- a/SimulationEngine/SimulationEngine/NeighborTest.xlsx
+++ b/SimulationEngine/SimulationEngine/NeighborTest.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\6-Courses\19-ModernC++Projects\SimulationEngine\SimulationEngine\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C50483B5-E871-49E8-ACCC-82301BC759E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5C2826C-E1B1-46A4-B9D5-13F51865B694}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{D5DDC3B4-E262-4B33-B762-D227AD5ACECE}"/>
   </bookViews>
@@ -966,7 +966,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F835845-E7D8-43A5-A30F-70FD886764B4}">
-  <dimension ref="A1:P15"/>
+  <dimension ref="A1:P23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.3">
@@ -1393,6 +1393,17 @@
     <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="H13">
         <v>70</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="K14">
+        <v>1</v>
+      </c>
+      <c r="L14">
+        <v>2</v>
+      </c>
+      <c r="M14">
+        <v>3</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.3">
@@ -1405,6 +1416,109 @@
         <f t="array" ref="H15">DIST(1,2)</f>
         <v>20.615528128088304</v>
       </c>
+      <c r="K15">
+        <v>2</v>
+      </c>
+      <c r="L15">
+        <v>1</v>
+      </c>
+      <c r="M15">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="K16">
+        <v>3</v>
+      </c>
+      <c r="L16">
+        <v>1</v>
+      </c>
+      <c r="M16">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="11:15" x14ac:dyDescent="0.3">
+      <c r="K17">
+        <v>4</v>
+      </c>
+      <c r="L17">
+        <v>5</v>
+      </c>
+      <c r="M17">
+        <v>6</v>
+      </c>
+      <c r="N17">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18" spans="11:15" x14ac:dyDescent="0.3">
+      <c r="K18">
+        <v>5</v>
+      </c>
+      <c r="L18">
+        <v>4</v>
+      </c>
+      <c r="M18">
+        <v>6</v>
+      </c>
+      <c r="N18">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19" spans="11:15" x14ac:dyDescent="0.3">
+      <c r="K19">
+        <v>6</v>
+      </c>
+      <c r="L19">
+        <v>4</v>
+      </c>
+      <c r="M19">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="11:15" x14ac:dyDescent="0.3">
+      <c r="K20">
+        <v>7</v>
+      </c>
+      <c r="L20">
+        <v>4</v>
+      </c>
+      <c r="M20">
+        <v>5</v>
+      </c>
+      <c r="N20">
+        <v>6</v>
+      </c>
+      <c r="O20">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21" spans="11:15" x14ac:dyDescent="0.3">
+      <c r="K21">
+        <v>8</v>
+      </c>
+      <c r="L21">
+        <v>6</v>
+      </c>
+      <c r="M21">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22" spans="11:15" x14ac:dyDescent="0.3">
+      <c r="K22">
+        <v>9</v>
+      </c>
+      <c r="L22">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="23" spans="11:15" x14ac:dyDescent="0.3">
+      <c r="K23">
+        <v>10</v>
+      </c>
+      <c r="L23">
+        <v>9</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Some refactoring and added a new test for the communicator
</commit_message>
<xml_diff>
--- a/SimulationEngine/SimulationEngine/NeighborTest.xlsx
+++ b/SimulationEngine/SimulationEngine/NeighborTest.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\6-Courses\19-ModernC++Projects\SimulationEngine\SimulationEngine\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5C2826C-E1B1-46A4-B9D5-13F51865B694}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{206610DB-B93D-4DCB-8471-B8D8825F4E68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{D5DDC3B4-E262-4B33-B762-D227AD5ACECE}"/>
+    <workbookView xWindow="-336" yWindow="2136" windowWidth="17916" windowHeight="10188" activeTab="1" xr2:uid="{D5DDC3B4-E262-4B33-B762-D227AD5ACECE}"/>
   </bookViews>
   <sheets>
     <sheet name="test1" sheetId="1" r:id="rId1"/>
@@ -1475,6 +1475,12 @@
       <c r="M19">
         <v>5</v>
       </c>
+      <c r="N19">
+        <v>7</v>
+      </c>
+      <c r="O19">
+        <v>8</v>
+      </c>
     </row>
     <row r="20" spans="11:15" x14ac:dyDescent="0.3">
       <c r="K20">

</xml_diff>